<commit_message>
integrated notification and real time fetching
</commit_message>
<xml_diff>
--- a/backend/data/customs_exit_with_est.xlsx
+++ b/backend/data/customs_exit_with_est.xlsx
@@ -236,7 +236,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="130">
+  <cellXfs count="132">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -621,6 +621,10 @@
     <xf numFmtId="167" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1018,7 +1022,11 @@
           <t>BL NUMBER</t>
         </is>
       </c>
-      <c r="P1" s="6" t="n"/>
+      <c r="P1" s="3" t="inlineStr">
+        <is>
+          <t>CHEQUE AMOUNT</t>
+        </is>
+      </c>
       <c r="Q1" s="6" t="n"/>
       <c r="R1" s="6" t="n"/>
       <c r="S1" s="6" t="n"/>
@@ -17271,7 +17279,7 @@
       <c r="F444" s="87" t="n"/>
       <c r="G444" s="88" t="inlineStr">
         <is>
-          <t>CONTAINER NO. MSMU3539604, MSDU 2817303, MSDU 1687798, MSDU 1027731, BEAU 2973978 -DICAM SARL</t>
+          <t>BEAU2973978, MSDU1027731, MSDU1687798, MSDU2817303, MSMU3539604</t>
         </is>
       </c>
       <c r="H444" s="88" t="n"/>
@@ -17285,10 +17293,24 @@
           <t>CARGOLINE</t>
         </is>
       </c>
-      <c r="K444" s="80" t="n"/>
-      <c r="L444" s="80" t="n"/>
-      <c r="M444" s="87" t="n"/>
-      <c r="N444" s="87" t="n"/>
+      <c r="K444" s="80" t="inlineStr">
+        <is>
+          <t>Mediterranean Shipping Company (MSC)</t>
+        </is>
+      </c>
+      <c r="L444" s="80" t="n">
+        <v>5</v>
+      </c>
+      <c r="M444" s="129" t="inlineStr">
+        <is>
+          <t>2026-10-03T00:00:00+04:00</t>
+        </is>
+      </c>
+      <c r="N444" s="129" t="inlineStr">
+        <is>
+          <t>2026-12-11T00:00:00+01:00</t>
+        </is>
+      </c>
       <c r="O444" s="96" t="inlineStr">
         <is>
           <t>MEDUH9299551</t>
@@ -21642,7 +21664,7 @@
       </c>
       <c r="G521" s="88" t="inlineStr">
         <is>
-          <t>GCXU2380730/CAIU6377190/GCXU2314446/TLLU2847114/CMAU0850652/BEAU2455789/</t>
+          <t>FCIU6239081, TLLU2000520, CMAU2856351, GLDU9953283, CAIU6377190, GCXU2380730, CMAU0850652, BEAU2455789, TLLU2847114, GCXU2314446</t>
         </is>
       </c>
       <c r="H521" s="88" t="inlineStr">
@@ -21662,22 +21684,29 @@
       </c>
       <c r="K521" s="114" t="inlineStr">
         <is>
-          <t>www.cma-cgm.com</t>
+          <t>CMA CGM</t>
         </is>
       </c>
       <c r="L521" s="119" t="n">
-        <v>6</v>
-      </c>
-      <c r="M521" s="119" t="n"/>
-      <c r="N521" s="87" t="inlineStr">
-        <is>
-          <t>14/1/2027</t>
+        <v>10</v>
+      </c>
+      <c r="M521" s="130" t="inlineStr">
+        <is>
+          <t>2026-10-25T00:00:00+04:00</t>
+        </is>
+      </c>
+      <c r="N521" s="129" t="inlineStr">
+        <is>
+          <t>2027-01-14T23:00:00+01:00</t>
         </is>
       </c>
       <c r="O521" s="96" t="inlineStr">
         <is>
           <t>DXB1062652</t>
         </is>
+      </c>
+      <c r="P521" s="131" t="n">
+        <v>2350.4</v>
       </c>
     </row>
     <row r="522" ht="15.75" customHeight="1" s="128">
@@ -21707,7 +21736,7 @@
       </c>
       <c r="G522" s="88" t="inlineStr">
         <is>
-          <t>GLDU9953283/CMAU2856351/TLLU2000520/FCIU6239081</t>
+          <t>FCIU6239081, TLLU2000520, CMAU2856351, GLDU9953283, CAIU6377190, GCXU2380730, CMAU0850652, BEAU2455789, TLLU2847114, GCXU2314446</t>
         </is>
       </c>
       <c r="H522" s="88" t="inlineStr">
@@ -21727,22 +21756,29 @@
       </c>
       <c r="K522" s="114" t="inlineStr">
         <is>
-          <t>www.cma-cgm.com</t>
+          <t>CMA CGM</t>
         </is>
       </c>
       <c r="L522" s="119" t="n">
-        <v>4</v>
-      </c>
-      <c r="M522" s="119" t="n"/>
-      <c r="N522" s="87" t="inlineStr">
-        <is>
-          <t>14/1/2027</t>
+        <v>10</v>
+      </c>
+      <c r="M522" s="130" t="inlineStr">
+        <is>
+          <t>2026-10-25T00:00:00+04:00</t>
+        </is>
+      </c>
+      <c r="N522" s="129" t="inlineStr">
+        <is>
+          <t>2027-01-14T23:00:00+01:00</t>
         </is>
       </c>
       <c r="O522" s="96" t="inlineStr">
         <is>
           <t>DXB1062652</t>
         </is>
+      </c>
+      <c r="P522" s="131" t="n">
+        <v>2350.4</v>
       </c>
     </row>
     <row r="523" ht="15.75" customHeight="1" s="128">

</xml_diff>